<commit_message>
Fix Trophy teammates when group_id equals phone number.
Auto-derive groups from participant ID (1A-6F → GROUP_N, staff → GROUP_STAFF).
Regenerate Excel template with correct group_id for all 49 participants.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/HKCYSTINTJustForYou_Sheet_Template.xlsx
+++ b/HKCYSTINTJustForYou_Sheet_Template.xlsx
@@ -786,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -819,12 +819,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>91234567</t>
+          <t>98765432</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>GROUP1</t>
+          <t>GROUP_1</t>
         </is>
       </c>
     </row>
@@ -836,93 +836,820 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>91234568</t>
+          <t>98765438</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>GROUP1</t>
+          <t>GROUP_1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>1C</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>91234569</t>
+          <t>98765444</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>GROUP2</t>
+          <t>GROUP_1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2B</t>
+          <t>1D</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>91234570</t>
+          <t>98765450</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>GROUP2</t>
+          <t>GROUP_1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>3A</t>
+          <t>1E</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>91234571</t>
+          <t>98765456</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>GROUP3</t>
+          <t>GROUP_1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
+          <t>1F</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>98765462</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>98765433</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>98765439</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2C</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>98765445</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2D</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>98765451</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2E</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>98765457</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2F</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>98765463</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>98765434</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>3B</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>91234572</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>GROUP3</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>說明：participant_id 為大寫（如 1A）。phone_number 僅數字。group_id 用於 Trophy 隊友分組。</t>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>98765440</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>3C</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>98765446</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>3D</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>98765452</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>3E</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>98765458</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>3F</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>98765464</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>98765435</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_4</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>98765441</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_4</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>4C</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>98765447</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_4</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>4D</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>98765453</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_4</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>4E</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>98765459</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_4</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>98765465</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_4</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>98765436</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>5B</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>98765442</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>5C</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>98765448</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>5D</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>98765454</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>5E</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>98765460</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>5F</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>98765466</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>6A</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>98765437</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_6</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>6B</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>98765443</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_6</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>6C</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>98765449</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_6</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>6D</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>98765455</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_6</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>6E</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>98765461</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_6</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>6F</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr"/>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_6</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>WILL</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>11111111</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>PHOEBE</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>22222222</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>RIGHT</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>33333333</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>RENAE</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>44444444</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>CHUNJAI</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>55555555</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>IRENE</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>66666666</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>KAKA</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>77777777</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>KAYI</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>88888888</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>WINGLAM</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>99999999</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>CHERYL</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>00000000</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>QQ</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>12121212</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>KELLY</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>13131313</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>BRO</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>14141414</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>GROUP_STAFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>說明：group_id 必須相同才能成為 Trophy 隊友。1A-1F 用 GROUP_1，2A-2F 用 GROUP_2… 工作人員用 GROUP_STAFF。勿將電話號碼填入 group_id！</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A52:F52"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>